<commit_message>
[rot][STiROT+OEMuROT] Fix issues of Loader and moficiations for STiROT + OEMuROT integration
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H553ZG/Applications/ROT/ROT_Flashlayout.xlsx
+++ b/Projects/NUCLEO-H553ZG/Applications/ROT/ROT_Flashlayout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ST\Cube\Cube1\STM32CubeH5\Projects\NUCLEO-H553ZG\Applications\ROT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D8F2D5-33EB-443B-B317-90CD0D783260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A25A2FD-0BD8-45FB-A2CA-23D34E4BC305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EA4F91E5-2F2C-41F9-ADC4-50A0D48CACE5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{EA4F91E5-2F2C-41F9-ADC4-50A0D48CACE5}"/>
   </bookViews>
   <sheets>
     <sheet name="OEMiROT+FullSec App Layout (2)" sheetId="5" r:id="rId1"/>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="54">
   <si>
     <t>FLASH_BASE</t>
   </si>
@@ -240,9 +240,6 @@
     <t>With this layout, there must be the download area of BL2 (OEMiROT + LOADER) in NS area (to be put at the end of the flash before EDATA area)</t>
   </si>
   <si>
-    <t>OEMiROT Downlaod</t>
-  </si>
-  <si>
     <t>Must be multiple of page size (2000), e.g. 4000</t>
   </si>
   <si>
@@ -253,6 +250,9 @@
   </si>
   <si>
     <t>This is fixed to 0x2000</t>
+  </si>
+  <si>
+    <t>OEMiROT FW Downlaod</t>
   </si>
 </sst>
 </file>
@@ -583,7 +583,27 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="20">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2457,34 +2477,34 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:B8 B10">
-    <cfRule type="cellIs" dxfId="17" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="7" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="8" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J30:J39">
-    <cfRule type="cellIs" dxfId="15" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16:M23">
-    <cfRule type="cellIs" dxfId="13" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="5" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="6" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K31:M39">
-    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2509,7 +2529,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00141F7F-4FCA-4FA8-9278-8A6044901D08}">
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
@@ -2737,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -2773,13 +2793,13 @@
     </row>
     <row r="14" spans="1:13" ht="16.5" customHeight="1">
       <c r="A14" s="36" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B14" s="6">
         <v>2000</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
@@ -3209,13 +3229,13 @@
     </row>
     <row r="25" spans="1:13">
       <c r="A25" s="12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C25" s="1" t="str">
-        <f>DEC2HEX(HEX2DEC($B$4)-HEX2DEC(F27)-HEX2DEC(F26)-HEX2DEC(F18))</f>
+      <c r="C25" s="12" t="str">
+        <f>DEC2HEX(HEX2DEC($B$4)-HEX2DEC(F27)-HEX2DEC(F26)-HEX2DEC(F25))</f>
         <v>DE000</v>
       </c>
       <c r="D25" s="1" t="str">
@@ -3224,23 +3244,23 @@
       </c>
       <c r="E25" s="1" t="str">
         <f t="shared" ref="E25:E27" si="7">DEC2HEX(HEX2DEC(D25)+HEX2DEC(F25)-1)</f>
-        <v>80FDFFF</v>
+        <v>80DFFFF</v>
       </c>
       <c r="F25" s="12">
-        <f>IF($B$13="Y",F18,0)</f>
-        <v>20000</v>
+        <f>IF($B$13="Y",$B$14,0)</f>
+        <v>2000</v>
       </c>
       <c r="G25" s="1">
         <f t="shared" ref="G25:G27" si="8">H25/1024</f>
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="H25" s="13">
         <f t="shared" ref="H25:H27" si="9">HEX2DEC(F25)</f>
-        <v>131072</v>
+        <v>8192</v>
       </c>
       <c r="I25" s="14">
         <f t="shared" ref="I25:I27" si="10">H25/HEX2DEC($B$5)</f>
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="J25" s="14" t="str">
         <f>$B$13</f>
@@ -3258,38 +3278,38 @@
     </row>
     <row r="26" spans="1:13">
       <c r="A26" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="1" t="str">
+      <c r="C26" s="12" t="str">
         <f>DEC2HEX(HEX2DEC($B$4)-HEX2DEC(F27)-HEX2DEC(F26))</f>
-        <v>FE000</v>
+        <v>E0000</v>
       </c>
       <c r="D26" s="1" t="str">
         <f t="shared" ref="D26" si="11">DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C26))</f>
-        <v>80FE000</v>
+        <v>80E0000</v>
       </c>
       <c r="E26" s="1" t="str">
         <f t="shared" ref="E26" si="12">DEC2HEX(HEX2DEC(D26)+HEX2DEC(F26)-1)</f>
         <v>80FFFFF</v>
       </c>
       <c r="F26" s="12">
-        <f>IF($B$13="Y",$B$14,0)</f>
-        <v>2000</v>
+        <f>IF($B$13="Y",F18,0)</f>
+        <v>20000</v>
       </c>
       <c r="G26" s="1">
         <f t="shared" ref="G26" si="13">H26/1024</f>
-        <v>8</v>
+        <v>128</v>
       </c>
       <c r="H26" s="13">
         <f t="shared" ref="H26" si="14">HEX2DEC(F26)</f>
-        <v>8192</v>
+        <v>131072</v>
       </c>
       <c r="I26" s="14">
         <f t="shared" ref="I26" si="15">H26/HEX2DEC($B$5)</f>
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="J26" s="14" t="str">
         <f>$B$13</f>
@@ -3511,15 +3531,15 @@
         <v>20000</v>
       </c>
       <c r="G35" s="1">
-        <f t="shared" ref="G35:G46" si="17">H35/1024</f>
+        <f t="shared" ref="G35:G48" si="17">H35/1024</f>
         <v>128</v>
       </c>
       <c r="H35" s="13">
-        <f t="shared" ref="H35:H43" si="18">HEX2DEC(F35)</f>
+        <f t="shared" ref="H35:H45" si="18">HEX2DEC(F35)</f>
         <v>131072</v>
       </c>
       <c r="I35" s="14">
-        <f t="shared" ref="I35:I43" si="19">H35/HEX2DEC($B$5)</f>
+        <f t="shared" ref="I35:I45" si="19">H35/HEX2DEC($B$5)</f>
         <v>16</v>
       </c>
       <c r="J35" s="14" t="s">
@@ -3645,11 +3665,11 @@
         <v>20000</v>
       </c>
       <c r="D38" s="1" t="str">
-        <f t="shared" ref="D38:D43" si="20">DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C38))</f>
+        <f t="shared" ref="D38:D45" si="20">DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C38))</f>
         <v>8020000</v>
       </c>
       <c r="E38" s="1" t="str">
-        <f t="shared" ref="E38:E43" si="21">DEC2HEX(HEX2DEC(D38)+HEX2DEC(F38)-1)</f>
+        <f t="shared" ref="E38:E45" si="21">DEC2HEX(HEX2DEC(D38)+HEX2DEC(F38)-1)</f>
         <v>801FFFF</v>
       </c>
       <c r="F38" s="1">
@@ -3844,23 +3864,23 @@
       </c>
       <c r="E42" s="33" t="str">
         <f t="shared" si="21"/>
-        <v>80FFFFF</v>
+        <v>80DDFFF</v>
       </c>
       <c r="F42" s="33" t="str">
         <f>DEC2HEX(HEX2DEC(C43)-HEX2DEC(C42))</f>
-        <v>CA000</v>
+        <v>A8000</v>
       </c>
       <c r="G42" s="33">
-        <f t="shared" ref="G42" si="23">H42/1024</f>
-        <v>808</v>
+        <f t="shared" ref="G42:G44" si="23">H42/1024</f>
+        <v>672</v>
       </c>
       <c r="H42" s="34">
-        <f t="shared" ref="H42" si="24">HEX2DEC(F42)</f>
-        <v>827392</v>
+        <f t="shared" ref="H42:H44" si="24">HEX2DEC(F42)</f>
+        <v>688128</v>
       </c>
       <c r="I42" s="35">
-        <f t="shared" ref="I42" si="25">H42/HEX2DEC($B$5)</f>
-        <v>101</v>
+        <f t="shared" ref="I42:I44" si="25">H42/HEX2DEC($B$5)</f>
+        <v>84</v>
       </c>
       <c r="J42" s="35"/>
       <c r="K42" s="35"/>
@@ -3869,176 +3889,282 @@
     </row>
     <row r="43" spans="1:13">
       <c r="A43" s="12" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C43" s="1" t="str">
-        <f>DEC2HEX(HEX2DEC($B$4)-HEX2DEC(F43))</f>
-        <v>100000</v>
+        <v>46</v>
+      </c>
+      <c r="C43" s="12" t="str">
+        <f>DEC2HEX(HEX2DEC($B$4)-HEX2DEC(F45)-HEX2DEC(F44)-HEX2DEC(F43))</f>
+        <v>DE000</v>
       </c>
       <c r="D43" s="1" t="str">
         <f t="shared" si="20"/>
-        <v>8100000</v>
+        <v>80DE000</v>
       </c>
       <c r="E43" s="1" t="str">
         <f t="shared" si="21"/>
+        <v>80DFFFF</v>
+      </c>
+      <c r="F43" s="12">
+        <f>IF($B$13="Y",$B$14,0)</f>
+        <v>2000</v>
+      </c>
+      <c r="G43" s="1">
+        <f t="shared" si="23"/>
+        <v>8</v>
+      </c>
+      <c r="H43" s="13">
+        <f t="shared" si="24"/>
+        <v>8192</v>
+      </c>
+      <c r="I43" s="14">
+        <f t="shared" si="25"/>
+        <v>1</v>
+      </c>
+      <c r="J43" s="14" t="str">
+        <f>$B$13</f>
+        <v>Y</v>
+      </c>
+      <c r="K43" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="L43" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="M43" s="14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13">
+      <c r="A44" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C44" s="12" t="str">
+        <f>DEC2HEX(HEX2DEC($B$4)-HEX2DEC(F45)-HEX2DEC(F44))</f>
+        <v>E0000</v>
+      </c>
+      <c r="D44" s="1" t="str">
+        <f t="shared" si="20"/>
+        <v>80E0000</v>
+      </c>
+      <c r="E44" s="1" t="str">
+        <f t="shared" si="21"/>
         <v>80FFFFF</v>
       </c>
-      <c r="F43" s="1">
+      <c r="F44" s="12">
+        <f>IF($B$13="Y",F35,0)</f>
+        <v>20000</v>
+      </c>
+      <c r="G44" s="1">
+        <f t="shared" si="23"/>
+        <v>128</v>
+      </c>
+      <c r="H44" s="13">
+        <f t="shared" si="24"/>
+        <v>131072</v>
+      </c>
+      <c r="I44" s="14">
+        <f t="shared" si="25"/>
+        <v>16</v>
+      </c>
+      <c r="J44" s="14" t="str">
+        <f>$B$13</f>
+        <v>Y</v>
+      </c>
+      <c r="K44" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="L44" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="M44" s="14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13">
+      <c r="A45" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C45" s="1" t="str">
+        <f>DEC2HEX(HEX2DEC($B$4)-HEX2DEC(F45))</f>
+        <v>100000</v>
+      </c>
+      <c r="D45" s="1" t="str">
+        <f t="shared" si="20"/>
+        <v>8100000</v>
+      </c>
+      <c r="E45" s="1" t="str">
+        <f t="shared" si="21"/>
+        <v>80FFFFF</v>
+      </c>
+      <c r="F45" s="1">
         <f>$B$12</f>
         <v>0</v>
       </c>
-      <c r="G43" s="1">
+      <c r="G45" s="1">
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-      <c r="H43" s="13">
+      <c r="H45" s="13">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="I43" s="14">
+      <c r="I45" s="14">
         <f t="shared" si="19"/>
         <v>0</v>
       </c>
-      <c r="J43" s="14" t="str">
+      <c r="J45" s="14" t="str">
         <f>IF($B$12=0,"N","Y")</f>
         <v>N</v>
       </c>
-      <c r="K43" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="L43" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="M43" s="14" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13">
-      <c r="A44" s="2" t="s">
+      <c r="K45" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="L45" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="M45" s="14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13">
+      <c r="A46" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="27" t="str">
-        <f>DEC2HEX(H44)</f>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="27" t="str">
+        <f>DEC2HEX(H46)</f>
         <v>100000</v>
       </c>
-      <c r="G44" s="2">
+      <c r="G46" s="2">
         <f t="shared" si="17"/>
         <v>1024</v>
       </c>
-      <c r="H44" s="28">
-        <f>SUM(H35:H43)-H36</f>
+      <c r="H46" s="28">
+        <f>SUM(H35:H45)-H36</f>
         <v>1048576</v>
       </c>
-      <c r="I44" s="5">
-        <f>H44/HEX2DEC($B$5)</f>
+      <c r="I46" s="5">
+        <f>H46/HEX2DEC($B$5)</f>
         <v>128</v>
-      </c>
-      <c r="J44" s="5"/>
-      <c r="K44" s="5"/>
-      <c r="L44" s="5"/>
-      <c r="M44" s="5"/>
-    </row>
-    <row r="45" spans="1:13">
-      <c r="A45" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="28">
-        <f>$B$4</f>
-        <v>100000</v>
-      </c>
-      <c r="G45" s="2">
-        <f t="shared" si="17"/>
-        <v>1024</v>
-      </c>
-      <c r="H45" s="28">
-        <f>HEX2DEC(F45)</f>
-        <v>1048576</v>
-      </c>
-      <c r="I45" s="5">
-        <f t="shared" ref="I45:I46" si="26">H45/HEX2DEC($B$5)</f>
-        <v>128</v>
-      </c>
-      <c r="J45" s="5"/>
-      <c r="K45" s="5"/>
-      <c r="L45" s="5"/>
-      <c r="M45" s="5"/>
-    </row>
-    <row r="46" spans="1:13">
-      <c r="A46" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="B46" s="5"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="28" t="str">
-        <f>DEC2HEX(H46)</f>
-        <v>0</v>
-      </c>
-      <c r="G46" s="2">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="H46" s="28">
-        <f>H45-H44</f>
-        <v>0</v>
-      </c>
-      <c r="I46" s="5">
-        <f t="shared" si="26"/>
-        <v>0</v>
       </c>
       <c r="J46" s="5"/>
       <c r="K46" s="5"/>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
     </row>
+    <row r="47" spans="1:13">
+      <c r="A47" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="28">
+        <f>$B$4</f>
+        <v>100000</v>
+      </c>
+      <c r="G47" s="2">
+        <f t="shared" si="17"/>
+        <v>1024</v>
+      </c>
+      <c r="H47" s="28">
+        <f>HEX2DEC(F47)</f>
+        <v>1048576</v>
+      </c>
+      <c r="I47" s="5">
+        <f t="shared" ref="I47:I48" si="26">H47/HEX2DEC($B$5)</f>
+        <v>128</v>
+      </c>
+      <c r="J47" s="5"/>
+      <c r="K47" s="5"/>
+      <c r="L47" s="5"/>
+      <c r="M47" s="5"/>
+    </row>
+    <row r="48" spans="1:13">
+      <c r="A48" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="28" t="str">
+        <f>DEC2HEX(H48)</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="2">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="H48" s="28">
+        <f>H47-H46</f>
+        <v>0</v>
+      </c>
+      <c r="I48" s="5">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5"/>
+      <c r="L48" s="5"/>
+      <c r="M48" s="5"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B6:B8 B10">
-    <cfRule type="cellIs" dxfId="9" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="29" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="30" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J34:J43">
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
+  <conditionalFormatting sqref="J34:J42 J45">
+    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="6" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J18:M27">
-    <cfRule type="cellIs" dxfId="5" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="19" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="20" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K35:M43">
-    <cfRule type="cellIs" dxfId="3" priority="15" operator="equal">
+  <conditionalFormatting sqref="K35:M42 K45:M45">
+    <cfRule type="cellIs" dxfId="5" priority="17" operator="equal">
       <formula>"N"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="18" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"Y"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J43:M44">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
@@ -4046,17 +4172,17 @@
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
-    <dataValidation type="decimal" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Total size consumed cannot exceed total user flash size!" sqref="H28 H44" xr:uid="{1A086C2B-0E4F-4241-80B5-5A1318638A48}">
+  <dataValidations disablePrompts="1" count="4">
+    <dataValidation type="decimal" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Total size consumed cannot exceed total user flash size!" sqref="H28 H46" xr:uid="{1A086C2B-0E4F-4241-80B5-5A1318638A48}">
       <formula1>H29</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10 B6:B8 B13 K35:M43 K18:M27" xr:uid="{1B61E276-0A20-47FF-BFB8-75ABA9EC3C08}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10 B6:B8 B13 K18:M27 K35:M45" xr:uid="{1B61E276-0A20-47FF-BFB8-75ABA9EC3C08}">
       <formula1>$B$1:$B$2</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="J18:J19 J35:J36" xr:uid="{55B1DDF0-6712-4B91-9618-826138437A1B}">
       <formula1>$B$1:$B$2</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F28 F44" xr:uid="{6EDCA1F8-9121-4096-AEAC-01BAB2B81477}">
+    <dataValidation type="whole" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F28 F46" xr:uid="{6EDCA1F8-9121-4096-AEAC-01BAB2B81477}">
       <formula1>F29</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>